<commit_message>
auto commit: 2026-03-20 09:43:48
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/测试用例/最终版测试用例/快乐羊毛系统完整测试用例2026.03.17（付仕菊）-V3.0完善版v2.xlsx
+++ b/快乐羊毛系统/测试用例/最终版测试用例/快乐羊毛系统完整测试用例2026.03.17（付仕菊）-V3.0完善版v2.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="13545" windowHeight="11925"/>
+    <workbookView windowWidth="27945" windowHeight="11925"/>
   </bookViews>
   <sheets>
     <sheet name="快乐羊毛测试用例" sheetId="1" r:id="rId1"/>
@@ -23888,7 +23888,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J453" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J44 A45:H45 J45 A46:J439 A440:E440 G440:J440 A441:J453" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>